<commit_message>
Update logistics sector (VDS_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/logistics sector (VDS_s) 0.xlsx
+++ b/clustering/sepsectors/logistics sector (VDS_s) 0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="21">
   <si>
     <t>sector</t>
   </si>
@@ -480,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="73.7109375" customWidth="1"/>
@@ -798,7 +798,7 @@
         <v>2210689.4932816424</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B17" s="5" t="s">
         <v>18</v>
       </c>
@@ -819,7 +819,7 @@
         <v>1.0712234055705171E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B18" s="5" t="s">
         <v>19</v>
       </c>
@@ -840,7 +840,7 @@
         <v>1.9714033377901509E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B20" s="5" t="s">
         <v>20</v>
       </c>
@@ -859,6 +859,362 @@
       <c r="G20" s="3">
         <f t="shared" si="2"/>
         <v>0.54338114633168244</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D23" s="3">
+        <v>4855346.2125374135</v>
+      </c>
+      <c r="E23" s="3">
+        <v>135386.12959937999</v>
+      </c>
+      <c r="F23" s="4">
+        <v>3.714330459169155E-3</v>
+      </c>
+      <c r="G23" s="4">
+        <v>1.653323199151599E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D24" s="3">
+        <v>4794949.4413491804</v>
+      </c>
+      <c r="E24" s="3">
+        <v>99309.261365249986</v>
+      </c>
+      <c r="F24" s="4">
+        <v>2.5245281739425698E-3</v>
+      </c>
+      <c r="G24" s="4">
+        <v>8.8733431342220078E-4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D25" s="3">
+        <v>4600808.5022977749</v>
+      </c>
+      <c r="E25" s="3">
+        <v>60802.035819069999</v>
+      </c>
+      <c r="F25" s="4">
+        <v>6.8489439848556958E-3</v>
+      </c>
+      <c r="G25" s="4">
+        <v>8.4462018431121508E-4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D26" s="3">
+        <v>4270265.7526510246</v>
+      </c>
+      <c r="E26" s="3">
+        <v>72255.755925899997</v>
+      </c>
+      <c r="F26" s="4">
+        <v>2.7888505476110981E-2</v>
+      </c>
+      <c r="G26" s="4">
+        <v>1.402683970588293E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D28" s="3">
+        <f>AVERAGE(D23:D24)</f>
+        <v>4825147.8269432969</v>
+      </c>
+      <c r="E28" s="3">
+        <f t="shared" ref="E28:G28" si="3">AVERAGE(E23:E24)</f>
+        <v>117347.69548231499</v>
+      </c>
+      <c r="F28" s="4">
+        <f t="shared" si="3"/>
+        <v>3.1194293165558622E-3</v>
+      </c>
+      <c r="G28" s="4">
+        <f t="shared" si="3"/>
+        <v>1.2703287562868999E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="3">
+        <f>AVERAGE(D25:D26)</f>
+        <v>4435537.1274743993</v>
+      </c>
+      <c r="E29" s="3">
+        <f t="shared" ref="E29:G29" si="4">AVERAGE(E25:E26)</f>
+        <v>66528.895872484994</v>
+      </c>
+      <c r="F29" s="4">
+        <f t="shared" si="4"/>
+        <v>1.7368724730483339E-2</v>
+      </c>
+      <c r="G29" s="4">
+        <f t="shared" si="4"/>
+        <v>1.123652077449754E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="3">
+        <f>D28/D29</f>
+        <v>1.0878384484836321</v>
+      </c>
+      <c r="E31" s="3">
+        <f t="shared" ref="E31:G31" si="5">E28/E29</f>
+        <v>1.7638605592859029</v>
+      </c>
+      <c r="F31" s="3">
+        <f t="shared" si="5"/>
+        <v>0.17960036588529976</v>
+      </c>
+      <c r="G31" s="3">
+        <f t="shared" si="5"/>
+        <v>1.1305356718336195</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D34" s="3">
+        <v>2292248.1387702548</v>
+      </c>
+      <c r="E34" s="3">
+        <v>34254.624294250003</v>
+      </c>
+      <c r="F34" s="4">
+        <v>1.595347631915882E-3</v>
+      </c>
+      <c r="G34" s="4">
+        <v>9.361237617013568E-4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D35" s="3">
+        <v>2266287.1009142809</v>
+      </c>
+      <c r="E35" s="3">
+        <v>31237.990653870002</v>
+      </c>
+      <c r="F35" s="4">
+        <v>4.7806163538082437E-3</v>
+      </c>
+      <c r="G35" s="4">
+        <v>7.032550042484375E-4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="2">
+        <v>2022</v>
+      </c>
+      <c r="D36" s="3">
+        <v>2155091.885649004</v>
+      </c>
+      <c r="E36" s="3">
+        <v>55489.055466000013</v>
+      </c>
+      <c r="F36" s="4">
+        <v>8.0723796852959749E-4</v>
+      </c>
+      <c r="G36" s="4">
+        <v>7.0553447782127363E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D37" s="3">
+        <v>1926632.816358228</v>
+      </c>
+      <c r="E37" s="3">
+        <v>70482.351956779996</v>
+      </c>
+      <c r="F37" s="4">
+        <v>1.720869178633199E-3</v>
+      </c>
+      <c r="G37" s="4">
+        <v>1.9771398616983161E-4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="3">
+        <f>AVERAGE(D34:D35)</f>
+        <v>2279267.6198422676</v>
+      </c>
+      <c r="E39" s="3">
+        <f t="shared" ref="E39:G39" si="6">AVERAGE(E34:E35)</f>
+        <v>32746.307474060002</v>
+      </c>
+      <c r="F39" s="4">
+        <f t="shared" si="6"/>
+        <v>3.1879819928620629E-3</v>
+      </c>
+      <c r="G39" s="4">
+        <f t="shared" si="6"/>
+        <v>8.196893829748972E-4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B40" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="3">
+        <f>AVERAGE(D36:D37)</f>
+        <v>2040862.3510036161</v>
+      </c>
+      <c r="E40" s="3">
+        <f t="shared" ref="E40:G40" si="7">AVERAGE(E36:E37)</f>
+        <v>62985.703711390001</v>
+      </c>
+      <c r="F40" s="4">
+        <f t="shared" si="7"/>
+        <v>1.2640535735813983E-3</v>
+      </c>
+      <c r="G40" s="4">
+        <f t="shared" si="7"/>
+        <v>3.6265293821912841E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C42" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D42" s="3">
+        <f>D39/D40</f>
+        <v>1.116815947298657</v>
+      </c>
+      <c r="E42" s="3">
+        <f t="shared" ref="E42:G42" si="8">E39/E40</f>
+        <v>0.51990063688275234</v>
+      </c>
+      <c r="F42" s="3">
+        <f t="shared" si="8"/>
+        <v>2.5220307584192545</v>
+      </c>
+      <c r="G42" s="3">
+        <f t="shared" si="8"/>
+        <v>0.22602584912178772</v>
       </c>
     </row>
   </sheetData>
@@ -866,6 +1222,198 @@
     <sortCondition descending="1" ref="D2:D13"/>
   </sortState>
   <conditionalFormatting sqref="D2:D13">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E13">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F13">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G13">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17:D18">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E18">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F17:F18">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:G18">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D23:D26">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23:E26">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F23:F26">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23:G26">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D28:D29">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E28:E29">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F28:F29">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G28:G29">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D34:D37">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -877,7 +1425,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E13">
+  <conditionalFormatting sqref="E34:E37">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -889,7 +1437,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F13">
+  <conditionalFormatting sqref="F34:F37">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -901,7 +1449,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G13">
+  <conditionalFormatting sqref="G34:G37">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -913,7 +1461,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D17:D18">
+  <conditionalFormatting sqref="D39:D40">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -925,7 +1473,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E18">
+  <conditionalFormatting sqref="E39:E40">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -937,7 +1485,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F17:F18">
+  <conditionalFormatting sqref="F39:F40">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -949,7 +1497,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G17:G18">
+  <conditionalFormatting sqref="G39:G40">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>